<commit_message>
update: belt shape and dock point
</commit_message>
<xml_diff>
--- a/Assets/Resources/Levels.xlsx
+++ b/Assets/Resources/Levels.xlsx
@@ -113,7 +113,7 @@
     <t xml:space="preserve">C</t>
   </si>
   <si>
-    <t xml:space="preserve">A
+    <t xml:space="preserve">A 
 90</t>
   </si>
   <si>
@@ -121,7 +121,7 @@
 90</t>
   </si>
   <si>
-    <t xml:space="preserve">C
+    <t xml:space="preserve">C 
 90</t>
   </si>
   <si>
@@ -324,12 +324,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1900,7 +1900,7 @@
       <c r="I17" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="J17" s="6" t="s">
+      <c r="J17" s="5" t="s">
         <v>26</v>
       </c>
       <c r="K17" s="5" t="s">
@@ -2104,7 +2104,7 @@
       <c r="B20" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D20" s="5" t="s">
@@ -2149,7 +2149,7 @@
       <c r="Q20" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="R20" s="6" t="s">
+      <c r="R20" s="5" t="s">
         <v>26</v>
       </c>
       <c r="S20" s="5" t="s">
@@ -2261,7 +2261,7 @@
         <v>26</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>26</v>
@@ -2294,7 +2294,7 @@
         <v>26</v>
       </c>
       <c r="P22" s="5" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>26</v>
@@ -2489,7 +2489,7 @@
         <v>26</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>26</v>
@@ -2519,7 +2519,7 @@
         <v>26</v>
       </c>
       <c r="P25" s="5" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>26</v>
@@ -3169,14 +3169,14 @@
       <c r="G34" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H34" s="6" t="s">
+      <c r="H34" s="5" t="s">
         <v>26</v>
       </c>
       <c r="I34" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J34" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="J34" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="K34" s="5" t="s">
         <v>26</v>
@@ -3184,7 +3184,7 @@
       <c r="L34" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="M34" s="6" t="s">
+      <c r="M34" s="5" t="s">
         <v>26</v>
       </c>
       <c r="N34" s="5" t="s">
@@ -3379,17 +3379,17 @@
       <c r="B37" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>26</v>
       </c>
       <c r="E37" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F37" s="5" t="s">
         <v>3</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>26</v>
@@ -3424,7 +3424,7 @@
       <c r="Q37" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="R37" s="6" t="s">
+      <c r="R37" s="5" t="s">
         <v>26</v>
       </c>
       <c r="S37" s="5" t="s">
@@ -3619,7 +3619,7 @@
       <c r="G40" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H40" s="6" t="s">
+      <c r="H40" s="5" t="s">
         <v>26</v>
       </c>
       <c r="I40" s="5" t="s">
@@ -3634,7 +3634,7 @@
       <c r="L40" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="M40" s="6" t="s">
+      <c r="M40" s="5" t="s">
         <v>26</v>
       </c>
       <c r="N40" s="5" t="s">
@@ -4983,7 +4983,7 @@
       <c r="K58" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="L58" s="7" t="s">
+      <c r="L58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="M58" s="5" t="s">
@@ -5106,8 +5106,8 @@
       <c r="B60" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C60" s="7" t="s">
-        <v>4</v>
+      <c r="C60" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>26</v>
@@ -5160,8 +5160,8 @@
       <c r="T60" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="U60" s="7" t="s">
-        <v>5</v>
+      <c r="U60" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="V60" s="5" t="s">
         <v>26</v>
@@ -5491,7 +5491,7 @@
         <v>26</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="G65" s="5" t="s">
         <v>26</v>
@@ -5527,7 +5527,7 @@
         <v>26</v>
       </c>
       <c r="R65" s="5" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="S65" s="5" t="s">
         <v>26</v>
@@ -6171,32 +6171,32 @@
       <c r="G74" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H74" s="7" t="s">
+      <c r="H74" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I74" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J74" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="I74" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="J74" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="K74" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="L74" s="7" t="s">
+      <c r="L74" s="6" t="s">
         <v>29</v>
       </c>
       <c r="M74" s="5" t="s">
         <v>26</v>
       </c>
       <c r="N74" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O74" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="P74" s="7" t="s">
-        <v>27</v>
+      <c r="P74" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="Q74" s="5" t="s">
         <v>26</v>
@@ -6381,18 +6381,18 @@
       <c r="B77" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C77" s="7" t="s">
+      <c r="C77" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F77" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D77" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E77" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F77" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="G77" s="5" t="s">
         <v>26</v>
       </c>
@@ -6427,7 +6427,7 @@
         <v>26</v>
       </c>
       <c r="R77" s="5" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="S77" s="5" t="s">
         <v>26</v>
@@ -6435,8 +6435,8 @@
       <c r="T77" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="U77" s="7" t="s">
-        <v>6</v>
+      <c r="U77" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="V77" s="5" t="s">
         <v>26</v>
@@ -6621,7 +6621,7 @@
       <c r="G80" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H80" s="7" t="s">
+      <c r="H80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="I80" s="5" t="s">
@@ -6645,7 +6645,7 @@
       <c r="O80" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="P80" s="7" t="s">
+      <c r="P80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="Q80" s="5" t="s">
@@ -7907,7 +7907,7 @@
       <c r="J97" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="K97" s="7" t="s">
+      <c r="K97" s="6" t="s">
         <v>26</v>
       </c>
       <c r="L97" s="5" t="s">
@@ -8033,8 +8033,8 @@
       <c r="B99" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C99" s="7" t="s">
-        <v>4</v>
+      <c r="C99" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>26</v>
@@ -8081,8 +8081,8 @@
       <c r="R99" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="S99" s="7" t="s">
-        <v>5</v>
+      <c r="S99" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="T99" s="5" t="s">
         <v>26</v>
@@ -8334,7 +8334,7 @@
         <v>26</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>26</v>
@@ -8370,7 +8370,7 @@
         <v>26</v>
       </c>
       <c r="O103" s="5" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="P103" s="5" t="s">
         <v>26</v>
@@ -8492,8 +8492,8 @@
       <c r="E105" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F105" s="7" t="s">
-        <v>30</v>
+      <c r="F105" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="G105" s="5" t="s">
         <v>26</v>
@@ -8642,8 +8642,8 @@
       <c r="E107" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F107" s="5" t="s">
-        <v>26</v>
+      <c r="F107" s="7" t="s">
+        <v>30</v>
       </c>
       <c r="G107" s="5" t="s">
         <v>26</v>
@@ -8792,7 +8792,7 @@
       <c r="E109" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F109" s="7" t="s">
+      <c r="F109" s="6" t="s">
         <v>31</v>
       </c>
       <c r="G109" s="5" t="s">
@@ -8942,8 +8942,8 @@
       <c r="E111" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F111" s="5" t="s">
-        <v>26</v>
+      <c r="F111" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="G111" s="5" t="s">
         <v>26</v>
@@ -9092,8 +9092,8 @@
       <c r="E113" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F113" s="7" t="s">
-        <v>32</v>
+      <c r="F113" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="G113" s="5" t="s">
         <v>26</v>
@@ -9234,7 +9234,7 @@
         <v>26</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>26</v>
@@ -9270,7 +9270,7 @@
         <v>26</v>
       </c>
       <c r="O115" s="5" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="P115" s="5" t="s">
         <v>26</v>
@@ -9533,8 +9533,8 @@
       <c r="B119" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C119" s="7" t="s">
-        <v>3</v>
+      <c r="C119" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>26</v>
@@ -9581,8 +9581,8 @@
       <c r="R119" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="S119" s="7" t="s">
-        <v>6</v>
+      <c r="S119" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="T119" s="5" t="s">
         <v>26</v>
@@ -9776,7 +9776,7 @@
       <c r="H122" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="I122" s="7" t="s">
+      <c r="I122" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J122" s="5" t="s">
@@ -9791,7 +9791,7 @@
       <c r="M122" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="N122" s="7" t="s">
+      <c r="N122" s="6" t="s">
         <v>26</v>
       </c>
       <c r="O122" s="5" t="s">

</xml_diff>